<commit_message>
SUMEC Mk5 Pro bom update
</commit_message>
<xml_diff>
--- a/main_hw/SUMEC_MK_V_Pro/SUMEC_MK_V_Pro.xlsx
+++ b/main_hw/SUMEC_MK_V_Pro/SUMEC_MK_V_Pro.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\MenMe\Documents\GitHub\Sumec-MiniSumo-HW\main_hw\SUMEC_MK_V_Pro\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B29A1C46-0C9C-4BAB-BEFA-211D53ECF45C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FD3DC606-EF6E-45A0-B861-8C470E42DFC6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="14616" xr2:uid="{1A39BB49-E988-4D6C-82B2-69211C58EAC0}"/>
   </bookViews>
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="164" uniqueCount="144">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="172" uniqueCount="152">
   <si>
     <t>Id</t>
   </si>
@@ -452,6 +452,30 @@
   </si>
   <si>
     <t>3.3uH, 2.2A, 1616</t>
+  </si>
+  <si>
+    <t>AP62301Z6-7, 5V</t>
+  </si>
+  <si>
+    <t>INA226AIDGSR</t>
+  </si>
+  <si>
+    <t>100R, 250mW, 0805, vishay</t>
+  </si>
+  <si>
+    <t>0R. 250mW, 0805, vishay</t>
+  </si>
+  <si>
+    <t>52.3k, 125mW, 0805, vishay</t>
+  </si>
+  <si>
+    <t>Buzzer 80dB</t>
+  </si>
+  <si>
+    <t>SPDT SW</t>
+  </si>
+  <si>
+    <t>2m, 500mW, 0805, yageo</t>
   </si>
 </sst>
 </file>
@@ -1435,7 +1459,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{A519A05D-972C-40DF-91E2-64A5DCA16E9E}">
-  <dimension ref="A1:G43"/>
+  <dimension ref="A1:G42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="7.44140625" customWidth="1"/>
@@ -1470,14 +1494,31 @@
       </c>
     </row>
     <row r="2" spans="1:7" x14ac:dyDescent="0.3">
-      <c r="G2" s="1"/>
+      <c r="A2">
+        <v>1</v>
+      </c>
+      <c r="B2" t="s">
+        <v>13</v>
+      </c>
+      <c r="C2" t="s">
+        <v>7</v>
+      </c>
+      <c r="D2">
+        <v>6</v>
+      </c>
+      <c r="E2" t="s">
+        <v>14</v>
+      </c>
+      <c r="F2" s="8" t="s">
+        <v>108</v>
+      </c>
     </row>
     <row r="3" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A3">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C3" t="s">
         <v>7</v>
@@ -1486,78 +1527,79 @@
         <v>6</v>
       </c>
       <c r="E3" t="s">
-        <v>14</v>
-      </c>
-      <c r="F3" s="8" t="s">
-        <v>108</v>
+        <v>12</v>
+      </c>
+      <c r="F3" s="9" t="s">
+        <v>112</v>
       </c>
     </row>
     <row r="4" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A4">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="B4" t="s">
-        <v>11</v>
+        <v>15</v>
       </c>
       <c r="C4" t="s">
         <v>7</v>
       </c>
       <c r="D4">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E4" t="s">
-        <v>12</v>
-      </c>
-      <c r="F4" s="9" t="s">
-        <v>112</v>
+        <v>16</v>
+      </c>
+      <c r="F4" s="8" t="s">
+        <v>109</v>
       </c>
     </row>
     <row r="5" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A5">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="B5" t="s">
-        <v>15</v>
+        <v>6</v>
       </c>
       <c r="C5" t="s">
         <v>7</v>
       </c>
       <c r="D5">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E5" t="s">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="F5" s="8" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
     </row>
     <row r="6" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A6">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="B6" t="s">
-        <v>6</v>
+        <v>9</v>
       </c>
       <c r="C6" t="s">
         <v>7</v>
       </c>
       <c r="D6">
-        <v>14</v>
+        <v>2</v>
       </c>
       <c r="E6" t="s">
-        <v>8</v>
-      </c>
-      <c r="F6" s="8" t="s">
-        <v>110</v>
-      </c>
+        <v>10</v>
+      </c>
+      <c r="F6" s="10" t="s">
+        <v>142</v>
+      </c>
+      <c r="G6" s="8"/>
     </row>
     <row r="7" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A7">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="B7" t="s">
-        <v>9</v>
+        <v>17</v>
       </c>
       <c r="C7" t="s">
         <v>7</v>
@@ -1566,76 +1608,79 @@
         <v>2</v>
       </c>
       <c r="E7" t="s">
-        <v>10</v>
-      </c>
-      <c r="F7" s="10" t="s">
-        <v>142</v>
-      </c>
-      <c r="G7" s="8"/>
+        <v>18</v>
+      </c>
+      <c r="F7" s="8" t="s">
+        <v>111</v>
+      </c>
     </row>
     <row r="8" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A8">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="B8" t="s">
-        <v>17</v>
+        <v>52</v>
       </c>
       <c r="C8" t="s">
-        <v>7</v>
+        <v>53</v>
       </c>
       <c r="D8">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E8" t="s">
-        <v>18</v>
-      </c>
-      <c r="F8" s="8" t="s">
-        <v>111</v>
+        <v>54</v>
+      </c>
+      <c r="F8" s="10" t="s">
+        <v>151</v>
       </c>
     </row>
     <row r="9" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A9">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="B9" t="s">
-        <v>52</v>
+        <v>55</v>
       </c>
       <c r="C9" t="s">
         <v>53</v>
       </c>
       <c r="D9">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E9" t="s">
-        <v>54</v>
+        <v>56</v>
+      </c>
+      <c r="F9" s="8" t="s">
+        <v>117</v>
       </c>
     </row>
     <row r="10" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A10">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="B10" t="s">
-        <v>55</v>
+        <v>57</v>
       </c>
       <c r="C10" t="s">
         <v>53</v>
       </c>
       <c r="D10">
-        <v>19</v>
+        <v>2</v>
       </c>
       <c r="E10" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="F10" s="8" t="s">
-        <v>117</v>
-      </c>
+        <v>118</v>
+      </c>
+      <c r="G10" s="8"/>
     </row>
     <row r="11" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A11">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B11" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="C11" t="s">
         <v>53</v>
@@ -1644,19 +1689,19 @@
         <v>2</v>
       </c>
       <c r="E11" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="F11" s="8" t="s">
-        <v>118</v>
-      </c>
-      <c r="G11" s="8"/>
+        <v>121</v>
+      </c>
+      <c r="G11" s="1"/>
     </row>
     <row r="12" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A12">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B12" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="C12" t="s">
         <v>53</v>
@@ -1665,19 +1710,18 @@
         <v>2</v>
       </c>
       <c r="E12" t="s">
-        <v>60</v>
-      </c>
-      <c r="F12" s="8" t="s">
-        <v>121</v>
-      </c>
-      <c r="G12" s="1"/>
+        <v>62</v>
+      </c>
+      <c r="F12" s="10" t="s">
+        <v>120</v>
+      </c>
     </row>
     <row r="13" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A13">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="B13" t="s">
-        <v>61</v>
+        <v>63</v>
       </c>
       <c r="C13" t="s">
         <v>53</v>
@@ -1686,77 +1730,80 @@
         <v>2</v>
       </c>
       <c r="E13" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="F13" s="10" t="s">
-        <v>120</v>
-      </c>
+        <v>148</v>
+      </c>
+      <c r="G13" s="8"/>
     </row>
     <row r="14" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A14">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="B14" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="C14" t="s">
         <v>53</v>
       </c>
       <c r="D14">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E14" t="s">
-        <v>64</v>
-      </c>
-      <c r="G14" s="8"/>
+        <v>66</v>
+      </c>
+      <c r="F14" s="11" t="s">
+        <v>122</v>
+      </c>
     </row>
     <row r="15" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A15">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="B15" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="C15" t="s">
         <v>53</v>
       </c>
       <c r="D15">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E15" t="s">
-        <v>66</v>
-      </c>
-      <c r="F15" s="11" t="s">
-        <v>122</v>
-      </c>
+        <v>68</v>
+      </c>
+      <c r="F15" s="8" t="s">
+        <v>116</v>
+      </c>
+      <c r="G15" s="8"/>
     </row>
     <row r="16" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A16">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="B16" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="C16" t="s">
         <v>53</v>
       </c>
       <c r="D16">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E16" t="s">
-        <v>68</v>
-      </c>
-      <c r="F16" s="8" t="s">
-        <v>116</v>
-      </c>
-      <c r="G16" s="8"/>
+        <v>70</v>
+      </c>
+      <c r="F16" s="10" t="s">
+        <v>146</v>
+      </c>
     </row>
     <row r="17" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A17">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="B17" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C17" t="s">
         <v>53</v>
@@ -1765,176 +1812,185 @@
         <v>1</v>
       </c>
       <c r="E17" t="s">
-        <v>70</v>
+        <v>72</v>
+      </c>
+      <c r="F17" s="10" t="s">
+        <v>147</v>
       </c>
     </row>
     <row r="18" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A18">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="B18" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="C18" t="s">
         <v>53</v>
       </c>
       <c r="D18">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="E18" t="s">
-        <v>72</v>
+        <v>74</v>
+      </c>
+      <c r="F18" s="8" t="s">
+        <v>119</v>
       </c>
     </row>
     <row r="19" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A19">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="B19" t="s">
-        <v>73</v>
+        <v>44</v>
       </c>
       <c r="C19" t="s">
-        <v>53</v>
+        <v>45</v>
       </c>
       <c r="D19">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E19" t="s">
-        <v>74</v>
-      </c>
-      <c r="F19" s="8" t="s">
-        <v>119</v>
-      </c>
+        <v>132</v>
+      </c>
+      <c r="F19" s="10" t="s">
+        <v>143</v>
+      </c>
+      <c r="G19" s="1"/>
     </row>
     <row r="20" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A20">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="B20" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="C20" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="D20">
         <v>1</v>
       </c>
       <c r="E20" t="s">
-        <v>132</v>
-      </c>
-      <c r="F20" s="10" t="s">
-        <v>143</v>
-      </c>
-      <c r="G20" s="1"/>
+        <v>48</v>
+      </c>
+      <c r="F20" s="8" t="s">
+        <v>114</v>
+      </c>
     </row>
     <row r="21" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A21">
+        <v>20</v>
+      </c>
+      <c r="B21" t="s">
         <v>19</v>
       </c>
-      <c r="B21" t="s">
-        <v>46</v>
-      </c>
       <c r="C21" t="s">
-        <v>47</v>
+        <v>20</v>
       </c>
       <c r="D21">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E21" t="s">
-        <v>48</v>
-      </c>
-      <c r="F21" s="8" t="s">
-        <v>114</v>
+        <v>21</v>
+      </c>
+      <c r="F21" s="10" t="s">
+        <v>135</v>
+      </c>
+      <c r="G21" s="10" t="s">
+        <v>136</v>
       </c>
     </row>
     <row r="22" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A22">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="B22" t="s">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="C22" t="s">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="D22">
-        <v>2</v>
+        <v>9</v>
       </c>
       <c r="E22" t="s">
-        <v>21</v>
-      </c>
-      <c r="F22" s="10" t="s">
-        <v>135</v>
+        <v>24</v>
       </c>
       <c r="G22" s="10" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
     </row>
     <row r="23" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A23">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="B23" t="s">
-        <v>22</v>
+        <v>79</v>
       </c>
       <c r="C23" t="s">
-        <v>23</v>
+        <v>80</v>
       </c>
       <c r="D23">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="E23" t="s">
-        <v>24</v>
+        <v>81</v>
+      </c>
+      <c r="F23" s="10" t="s">
+        <v>145</v>
       </c>
       <c r="G23" s="10" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
     </row>
     <row r="24" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A24">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="B24" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C24" t="s">
-        <v>80</v>
+        <v>83</v>
       </c>
       <c r="D24">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E24" t="s">
-        <v>81</v>
-      </c>
-      <c r="G24" s="10" t="s">
-        <v>138</v>
+        <v>84</v>
+      </c>
+      <c r="F24" s="10" t="s">
+        <v>83</v>
       </c>
     </row>
     <row r="25" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A25">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B25" t="s">
-        <v>82</v>
+        <v>85</v>
       </c>
       <c r="C25" t="s">
-        <v>83</v>
+        <v>86</v>
       </c>
       <c r="D25">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E25" t="s">
-        <v>84</v>
+        <v>87</v>
       </c>
       <c r="F25" s="10" t="s">
-        <v>83</v>
+        <v>144</v>
       </c>
     </row>
     <row r="26" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A26">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="B26" t="s">
-        <v>85</v>
+        <v>88</v>
       </c>
       <c r="C26" t="s">
         <v>86</v>
@@ -1943,376 +1999,373 @@
         <v>1</v>
       </c>
       <c r="E26" t="s">
-        <v>87</v>
+        <v>89</v>
+      </c>
+      <c r="F26" s="8" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="27" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A27">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="B27" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="C27" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="D27">
         <v>1</v>
       </c>
       <c r="E27" t="s">
-        <v>89</v>
+        <v>92</v>
       </c>
       <c r="F27" s="8" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
     </row>
     <row r="28" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A28">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="B28" t="s">
-        <v>90</v>
+        <v>93</v>
       </c>
       <c r="C28" t="s">
-        <v>91</v>
+        <v>94</v>
       </c>
       <c r="D28">
         <v>1</v>
       </c>
       <c r="E28" t="s">
-        <v>92</v>
+        <v>95</v>
       </c>
       <c r="F28" s="8" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
     </row>
     <row r="29" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A29">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="B29" t="s">
-        <v>93</v>
+        <v>96</v>
       </c>
       <c r="C29" t="s">
-        <v>94</v>
+        <v>97</v>
       </c>
       <c r="D29">
         <v>1</v>
       </c>
       <c r="E29" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="F29" s="8" t="s">
-        <v>125</v>
-      </c>
-      <c r="G29" s="10" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
     </row>
     <row r="30" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A30">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="B30" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="C30" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="D30">
         <v>1</v>
       </c>
       <c r="E30" t="s">
-        <v>97</v>
+        <v>100</v>
       </c>
       <c r="F30" s="8" t="s">
-        <v>128</v>
-      </c>
+        <v>124</v>
+      </c>
+      <c r="G30" s="8"/>
     </row>
     <row r="31" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A31">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="B31" t="s">
-        <v>98</v>
+        <v>49</v>
       </c>
       <c r="C31" t="s">
-        <v>99</v>
+        <v>50</v>
       </c>
       <c r="D31">
         <v>1</v>
       </c>
       <c r="E31" t="s">
-        <v>100</v>
+        <v>51</v>
       </c>
       <c r="F31" s="8" t="s">
-        <v>124</v>
-      </c>
-      <c r="G31" s="8"/>
+        <v>115</v>
+      </c>
     </row>
     <row r="32" spans="1:7" x14ac:dyDescent="0.3">
       <c r="A32">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="B32" t="s">
-        <v>49</v>
+        <v>3</v>
       </c>
       <c r="C32" t="s">
-        <v>50</v>
+        <v>4</v>
       </c>
       <c r="D32">
         <v>1</v>
       </c>
       <c r="E32" t="s">
-        <v>51</v>
-      </c>
-      <c r="F32" s="8" t="s">
-        <v>115</v>
+        <v>5</v>
+      </c>
+      <c r="F32" s="10" t="s">
+        <v>149</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33">
-        <v>31</v>
+        <v>32</v>
       </c>
       <c r="B33" t="s">
-        <v>3</v>
+        <v>101</v>
       </c>
       <c r="C33" t="s">
-        <v>4</v>
+        <v>102</v>
       </c>
       <c r="D33">
         <v>1</v>
       </c>
       <c r="E33" t="s">
-        <v>5</v>
+        <v>103</v>
+      </c>
+      <c r="F33" s="8" t="s">
+        <v>129</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="B34" t="s">
-        <v>101</v>
+        <v>75</v>
       </c>
       <c r="C34" t="s">
-        <v>102</v>
+        <v>76</v>
       </c>
       <c r="D34">
         <v>1</v>
       </c>
       <c r="E34" t="s">
-        <v>103</v>
-      </c>
-      <c r="F34" s="8" t="s">
-        <v>129</v>
+        <v>77</v>
+      </c>
+      <c r="F34" s="10" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="B35" t="s">
-        <v>75</v>
+        <v>130</v>
       </c>
       <c r="C35" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="D35">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="E35" t="s">
-        <v>77</v>
+        <v>131</v>
+      </c>
+      <c r="F35" s="8" t="s">
+        <v>123</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="B36" t="s">
-        <v>130</v>
+        <v>25</v>
       </c>
       <c r="C36" t="s">
-        <v>78</v>
+        <v>26</v>
       </c>
       <c r="D36">
-        <v>5</v>
+        <v>1</v>
       </c>
       <c r="E36" t="s">
-        <v>131</v>
-      </c>
-      <c r="F36" s="8" t="s">
-        <v>123</v>
+        <v>26</v>
+      </c>
+      <c r="F36" s="10" t="s">
+        <v>133</v>
       </c>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="B37" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="C37" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="D37">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E37" t="s">
-        <v>26</v>
+        <v>29</v>
       </c>
       <c r="F37" s="10" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="B38" t="s">
-        <v>27</v>
+        <v>30</v>
       </c>
       <c r="C38" t="s">
-        <v>28</v>
+        <v>31</v>
       </c>
       <c r="D38">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E38" t="s">
-        <v>29</v>
+        <v>32</v>
+      </c>
+      <c r="F38" s="8" t="s">
+        <v>113</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="B39" t="s">
-        <v>30</v>
+        <v>33</v>
       </c>
       <c r="C39" t="s">
-        <v>31</v>
+        <v>34</v>
       </c>
       <c r="D39">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="E39" t="s">
-        <v>32</v>
-      </c>
-      <c r="F39" s="8" t="s">
-        <v>113</v>
+        <v>35</v>
+      </c>
+      <c r="F39" s="10" t="s">
+        <v>140</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="s">
+        <v>36</v>
+      </c>
+      <c r="C40" t="s">
+        <v>37</v>
+      </c>
+      <c r="D40">
+        <v>1</v>
+      </c>
+      <c r="E40" t="s">
         <v>38</v>
       </c>
-      <c r="B40" t="s">
-        <v>33</v>
-      </c>
-      <c r="C40" t="s">
-        <v>34</v>
-      </c>
-      <c r="D40">
-        <v>6</v>
-      </c>
-      <c r="E40" t="s">
-        <v>35</v>
-      </c>
       <c r="F40" s="10" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="s">
         <v>39</v>
       </c>
-      <c r="B41" t="s">
-        <v>36</v>
-      </c>
       <c r="C41" t="s">
-        <v>37</v>
+        <v>40</v>
       </c>
       <c r="D41">
         <v>1</v>
       </c>
       <c r="E41" t="s">
-        <v>38</v>
+        <v>41</v>
       </c>
       <c r="F41" s="10" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="B42" t="s">
-        <v>39</v>
+        <v>42</v>
       </c>
       <c r="C42" t="s">
-        <v>40</v>
+        <v>43</v>
       </c>
       <c r="D42">
         <v>1</v>
       </c>
       <c r="E42" t="s">
-        <v>41</v>
-      </c>
-      <c r="F42" s="10" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A43">
-        <v>41</v>
-      </c>
-      <c r="B43" t="s">
-        <v>42</v>
-      </c>
-      <c r="C43" t="s">
-        <v>43</v>
-      </c>
-      <c r="D43">
-        <v>1</v>
-      </c>
-      <c r="E43" t="s">
         <v>35</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F3" r:id="rId1" xr:uid="{70F3D70B-444E-4EA0-93A6-FB8B4C314A91}"/>
-    <hyperlink ref="F5" r:id="rId2" xr:uid="{EF5F496A-8AEB-4870-84EF-6FD1FA2A442B}"/>
-    <hyperlink ref="F6" r:id="rId3" display="100nF, 16V, 0805, ceramic, mouser X7R" xr:uid="{394C0BFD-D893-4BEE-8875-6F800931C010}"/>
-    <hyperlink ref="F8" r:id="rId4" xr:uid="{7B9DD6E4-E929-4C6E-9F45-74F94CDB2673}"/>
-    <hyperlink ref="F4" r:id="rId5" display="0805, 10u, X7R, 16V, 10%, mouser" xr:uid="{1A574FFC-A94A-42B2-B18D-8C14D61195E4}"/>
-    <hyperlink ref="F39" r:id="rId6" xr:uid="{DA32D265-5AD9-4864-BFB0-7A2A7818BB06}"/>
-    <hyperlink ref="F21" r:id="rId7" xr:uid="{43F2BBC7-DA59-438B-A89B-0C646DB5CF91}"/>
-    <hyperlink ref="F32" r:id="rId8" xr:uid="{61CFA6D3-498F-4F8E-A435-764662CA774C}"/>
-    <hyperlink ref="F16" r:id="rId9" display="15R mouser" xr:uid="{95E9ED0F-1CB1-4E62-98F9-87361FF458E0}"/>
-    <hyperlink ref="F10" r:id="rId10" display="10k mouser" xr:uid="{E2E588A7-40B5-4000-BCA9-C2C50A43D430}"/>
-    <hyperlink ref="F12" r:id="rId11" display="100k, 250mW, 0805" xr:uid="{35202CB2-579A-405D-840F-B1A6EEE0FBD2}"/>
-    <hyperlink ref="F19" r:id="rId12" display="220R 250mW" xr:uid="{90BEC547-AE98-45DE-AFEA-D3235741B10C}"/>
-    <hyperlink ref="F15" r:id="rId13" display="45.3k, 125mW, vishay" xr:uid="{D3B8D38B-E4B9-4D72-9CFF-627D78391DDA}"/>
-    <hyperlink ref="F31" r:id="rId14" display="24CW1280T-I/OT EEPROMe" xr:uid="{DB9011EE-3E12-4D56-AE8D-CB0222D415C8}"/>
-    <hyperlink ref="F30" r:id="rId15" xr:uid="{D3926DBC-A7C8-4455-8D24-B7A7A4FB137E}"/>
-    <hyperlink ref="F36" r:id="rId16" xr:uid="{869105E7-048F-4332-9B4A-61CFF449970C}"/>
-    <hyperlink ref="F29" r:id="rId17" xr:uid="{6B208BCF-3B7C-4BEB-982B-CED8DF74013F}"/>
-    <hyperlink ref="F27" r:id="rId18" xr:uid="{422FB489-B301-4200-9D12-0E60F3147A01}"/>
-    <hyperlink ref="F34" r:id="rId19" xr:uid="{E631D7BC-568D-459E-A612-F33533B803FA}"/>
-    <hyperlink ref="F11" r:id="rId20" xr:uid="{CFE0BA31-58C3-49E8-90D2-075BA2FC8A41}"/>
-    <hyperlink ref="F13" r:id="rId21" xr:uid="{F43DD01B-1AD8-49FA-B605-1430DAE5F41B}"/>
-    <hyperlink ref="F37" r:id="rId22" xr:uid="{DD2581AE-A248-4009-B6D8-C74391BF1468}"/>
-    <hyperlink ref="G29" r:id="rId23" xr:uid="{873B68C9-1BB9-4D11-A582-FFF028D6A6D4}"/>
-    <hyperlink ref="F22" r:id="rId24" xr:uid="{E7BCAF4A-1605-43DC-AADC-B04D18173BC3}"/>
-    <hyperlink ref="G24" r:id="rId25" display="Red LED, 20mA 1.9V, 0805, mouser" xr:uid="{F0E2D0D5-8297-4922-8DF4-ED0B3D730DD5}"/>
-    <hyperlink ref="G22" r:id="rId26" display="Yellow LED, 20mA, 1.9V, 0805, mouser" xr:uid="{4A1ECE38-296B-4E90-B97E-C090FAAB478D}"/>
-    <hyperlink ref="G23" r:id="rId27" display="Green-Yellow LED, 20mA, 1.9V, mouser" xr:uid="{B9F382DE-A625-48FF-9A2D-726B40163E55}"/>
-    <hyperlink ref="F42" r:id="rId28" xr:uid="{C08E846E-85E7-4DED-863E-B8497898F762}"/>
-    <hyperlink ref="F40" r:id="rId29" xr:uid="{16E6A351-404B-4DFE-A26D-3745EE3F6515}"/>
-    <hyperlink ref="F41" r:id="rId30" xr:uid="{26DE56BE-6FDE-4A3E-824A-64A0E7BC8793}"/>
-    <hyperlink ref="F7" r:id="rId31" display="22nF, 50V, 0805, mouser, X7R" xr:uid="{FD883FC5-5954-4350-9EF5-178E847AA973}"/>
-    <hyperlink ref="F25" r:id="rId32" display="DRV8874.  mouser" xr:uid="{75667A55-2CCF-40B9-95A9-1A358EC72464}"/>
-    <hyperlink ref="F20" r:id="rId33" xr:uid="{B17139F4-D33A-4431-953B-2EDE67D3839C}"/>
+    <hyperlink ref="F2" r:id="rId1" xr:uid="{70F3D70B-444E-4EA0-93A6-FB8B4C314A91}"/>
+    <hyperlink ref="F4" r:id="rId2" xr:uid="{EF5F496A-8AEB-4870-84EF-6FD1FA2A442B}"/>
+    <hyperlink ref="F5" r:id="rId3" display="100nF, 16V, 0805, ceramic, mouser X7R" xr:uid="{394C0BFD-D893-4BEE-8875-6F800931C010}"/>
+    <hyperlink ref="F7" r:id="rId4" xr:uid="{7B9DD6E4-E929-4C6E-9F45-74F94CDB2673}"/>
+    <hyperlink ref="F3" r:id="rId5" display="0805, 10u, X7R, 16V, 10%, mouser" xr:uid="{1A574FFC-A94A-42B2-B18D-8C14D61195E4}"/>
+    <hyperlink ref="F38" r:id="rId6" xr:uid="{DA32D265-5AD9-4864-BFB0-7A2A7818BB06}"/>
+    <hyperlink ref="F20" r:id="rId7" xr:uid="{43F2BBC7-DA59-438B-A89B-0C646DB5CF91}"/>
+    <hyperlink ref="F31" r:id="rId8" xr:uid="{61CFA6D3-498F-4F8E-A435-764662CA774C}"/>
+    <hyperlink ref="F15" r:id="rId9" display="15R mouser" xr:uid="{95E9ED0F-1CB1-4E62-98F9-87361FF458E0}"/>
+    <hyperlink ref="F9" r:id="rId10" display="10k mouser" xr:uid="{E2E588A7-40B5-4000-BCA9-C2C50A43D430}"/>
+    <hyperlink ref="F11" r:id="rId11" display="100k, 250mW, 0805" xr:uid="{35202CB2-579A-405D-840F-B1A6EEE0FBD2}"/>
+    <hyperlink ref="F18" r:id="rId12" display="220R 250mW" xr:uid="{90BEC547-AE98-45DE-AFEA-D3235741B10C}"/>
+    <hyperlink ref="F14" r:id="rId13" display="45.3k, 125mW, vishay" xr:uid="{D3B8D38B-E4B9-4D72-9CFF-627D78391DDA}"/>
+    <hyperlink ref="F30" r:id="rId14" display="24CW1280T-I/OT EEPROMe" xr:uid="{DB9011EE-3E12-4D56-AE8D-CB0222D415C8}"/>
+    <hyperlink ref="F29" r:id="rId15" xr:uid="{D3926DBC-A7C8-4455-8D24-B7A7A4FB137E}"/>
+    <hyperlink ref="F35" r:id="rId16" xr:uid="{869105E7-048F-4332-9B4A-61CFF449970C}"/>
+    <hyperlink ref="F28" r:id="rId17" xr:uid="{6B208BCF-3B7C-4BEB-982B-CED8DF74013F}"/>
+    <hyperlink ref="F26" r:id="rId18" xr:uid="{422FB489-B301-4200-9D12-0E60F3147A01}"/>
+    <hyperlink ref="F33" r:id="rId19" xr:uid="{E631D7BC-568D-459E-A612-F33533B803FA}"/>
+    <hyperlink ref="F10" r:id="rId20" xr:uid="{CFE0BA31-58C3-49E8-90D2-075BA2FC8A41}"/>
+    <hyperlink ref="F12" r:id="rId21" xr:uid="{F43DD01B-1AD8-49FA-B605-1430DAE5F41B}"/>
+    <hyperlink ref="F36" r:id="rId22" xr:uid="{DD2581AE-A248-4009-B6D8-C74391BF1468}"/>
+    <hyperlink ref="F37" r:id="rId23" xr:uid="{873B68C9-1BB9-4D11-A582-FFF028D6A6D4}"/>
+    <hyperlink ref="F21" r:id="rId24" xr:uid="{E7BCAF4A-1605-43DC-AADC-B04D18173BC3}"/>
+    <hyperlink ref="G23" r:id="rId25" display="Red LED, 20mA 1.9V, 0805, mouser" xr:uid="{F0E2D0D5-8297-4922-8DF4-ED0B3D730DD5}"/>
+    <hyperlink ref="G21" r:id="rId26" display="Yellow LED, 20mA, 1.9V, 0805, mouser" xr:uid="{4A1ECE38-296B-4E90-B97E-C090FAAB478D}"/>
+    <hyperlink ref="G22" r:id="rId27" display="Green-Yellow LED, 20mA, 1.9V, mouser" xr:uid="{B9F382DE-A625-48FF-9A2D-726B40163E55}"/>
+    <hyperlink ref="F41" r:id="rId28" xr:uid="{C08E846E-85E7-4DED-863E-B8497898F762}"/>
+    <hyperlink ref="F39" r:id="rId29" xr:uid="{16E6A351-404B-4DFE-A26D-3745EE3F6515}"/>
+    <hyperlink ref="F40" r:id="rId30" xr:uid="{26DE56BE-6FDE-4A3E-824A-64A0E7BC8793}"/>
+    <hyperlink ref="F6" r:id="rId31" display="22nF, 50V, 0805, mouser, X7R" xr:uid="{FD883FC5-5954-4350-9EF5-178E847AA973}"/>
+    <hyperlink ref="F24" r:id="rId32" display="DRV8874.  mouser" xr:uid="{75667A55-2CCF-40B9-95A9-1A358EC72464}"/>
+    <hyperlink ref="F19" r:id="rId33" xr:uid="{B17139F4-D33A-4431-953B-2EDE67D3839C}"/>
+    <hyperlink ref="F25" r:id="rId34" xr:uid="{9A419603-1E3E-4170-BB81-F5465FF66777}"/>
+    <hyperlink ref="F23" r:id="rId35" display="INA226" xr:uid="{B7E2BEFB-9AE5-49CD-95E1-85FCAD810760}"/>
+    <hyperlink ref="F16" r:id="rId36" display="100R, 250mW, 0805" xr:uid="{A45E8C47-9205-4D3D-93D4-7C8D28F21F68}"/>
+    <hyperlink ref="F17" r:id="rId37" display="0R. 250mW, 0805" xr:uid="{A1DCDA25-89E7-4451-8D6D-E142B5208749}"/>
+    <hyperlink ref="F13" r:id="rId38" xr:uid="{87AD705C-A8E9-49DF-81EE-2CFDAD5C26E5}"/>
+    <hyperlink ref="F32" r:id="rId39" xr:uid="{5684D214-0F7B-47BB-B50F-4D2964C24C48}"/>
+    <hyperlink ref="F34" r:id="rId40" xr:uid="{38CAE819-5590-4344-AC0F-E30E907C8156}"/>
+    <hyperlink ref="F8" r:id="rId41" xr:uid="{9E903C02-E521-421B-B465-3F3247F81BB0}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.78740157499999996" bottom="0.78740157499999996" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>